<commit_message>
weekly commit after report generation for the week
</commit_message>
<xml_diff>
--- a/3_output/2026/w37/y2026_w37_weekly_report_output.xlsx
+++ b/3_output/2026/w37/y2026_w37_weekly_report_output.xlsx
@@ -3097,7 +3097,7 @@
         <v>0</v>
       </c>
       <c r="D26" s="26" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="E26" s="16" t="n">
         <v>0</v>
@@ -3115,7 +3115,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="26" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="K26" s="16" t="n">
         <v>0</v>
@@ -3160,7 +3160,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="26" t="n">
-        <v>0.08</v>
+        <v>0.07</v>
       </c>
       <c r="E27" s="16" t="n">
         <v>0.08</v>
@@ -3178,7 +3178,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="26" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="K27" s="16" t="n">
         <v>0.02</v>
@@ -3223,7 +3223,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="26" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="E28" s="16" t="n">
         <v>0</v>
@@ -3286,7 +3286,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="26" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="E29" s="16" t="n">
         <v>0.06</v>
@@ -3304,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="J29" s="26" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="K29" s="16" t="n">
         <v>0.01</v>
@@ -3349,7 +3349,7 @@
         <v>0</v>
       </c>
       <c r="D30" s="26" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="E30" s="16" t="n">
         <v>0.05</v>
@@ -3412,7 +3412,7 @@
         <v>0</v>
       </c>
       <c r="D31" s="26" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="E31" s="16" t="n">
         <v>0</v>
@@ -3430,7 +3430,7 @@
         <v>0.09</v>
       </c>
       <c r="J31" s="26" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="K31" s="16" t="n">
         <v>0.05</v>
@@ -6701,7 +6701,7 @@
         <v>0</v>
       </c>
       <c r="J92" s="14" t="n">
-        <v>1.3</v>
+        <v>1.24</v>
       </c>
       <c r="K92" s="14" t="n">
         <v>0</v>
@@ -6746,7 +6746,7 @@
         <v>0</v>
       </c>
       <c r="D93" s="14" t="n">
-        <v>2.38</v>
+        <v>2.5</v>
       </c>
       <c r="E93" s="14" t="n">
         <v>0</v>
@@ -6764,7 +6764,7 @@
         <v>0</v>
       </c>
       <c r="J93" s="14" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="K93" s="14" t="n">
         <v>0</v>
@@ -6809,7 +6809,7 @@
         <v>0</v>
       </c>
       <c r="D94" s="14" t="n">
-        <v>1.62</v>
+        <v>1.4</v>
       </c>
       <c r="E94" s="14" t="n">
         <v>1.3</v>
@@ -6827,7 +6827,7 @@
         <v>0</v>
       </c>
       <c r="J94" s="14" t="n">
-        <v>2.92</v>
+        <v>3.06</v>
       </c>
       <c r="K94" s="14" t="n">
         <v>0.8</v>
@@ -6872,7 +6872,7 @@
         <v>0</v>
       </c>
       <c r="D95" s="14" t="n">
-        <v>6.34</v>
+        <v>6.26</v>
       </c>
       <c r="E95" s="14" t="n">
         <v>0</v>
@@ -6890,7 +6890,7 @@
         <v>0</v>
       </c>
       <c r="J95" s="14" t="n">
-        <v>6.3</v>
+        <v>6.26</v>
       </c>
       <c r="K95" s="14" t="n">
         <v>0</v>
@@ -6935,7 +6935,7 @@
         <v>0</v>
       </c>
       <c r="D96" s="14" t="n">
-        <v>10.46</v>
+        <v>12.38</v>
       </c>
       <c r="E96" s="14" t="n">
         <v>1.1</v>
@@ -6953,7 +6953,7 @@
         <v>0</v>
       </c>
       <c r="J96" s="14" t="n">
-        <v>10.34</v>
+        <v>7.18</v>
       </c>
       <c r="K96" s="14" t="n">
         <v>0.6</v>
@@ -6998,7 +6998,7 @@
         <v>0</v>
       </c>
       <c r="D97" s="14" t="n">
-        <v>10.84</v>
+        <v>10.88</v>
       </c>
       <c r="E97" s="14" t="n">
         <v>1.1</v>
@@ -7016,7 +7016,7 @@
         <v>0</v>
       </c>
       <c r="J97" s="14" t="n">
-        <v>12.12</v>
+        <v>12.2</v>
       </c>
       <c r="K97" s="14" t="n">
         <v>1.1</v>
@@ -7061,7 +7061,7 @@
         <v>0</v>
       </c>
       <c r="D98" s="14" t="n">
-        <v>12.74</v>
+        <v>12.62</v>
       </c>
       <c r="E98" s="14" t="n">
         <v>0</v>
@@ -7079,7 +7079,7 @@
         <v>6.7</v>
       </c>
       <c r="J98" s="14" t="n">
-        <v>17.48</v>
+        <v>18.12</v>
       </c>
       <c r="K98" s="14" t="n">
         <v>2.8</v>
@@ -7124,7 +7124,7 @@
         <v>19.4</v>
       </c>
       <c r="D99" s="14" t="n">
-        <v>5.02</v>
+        <v>6.46</v>
       </c>
       <c r="E99" s="14" t="n">
         <v>1.8</v>
@@ -7142,7 +7142,7 @@
         <v>0</v>
       </c>
       <c r="J99" s="14" t="n">
-        <v>15</v>
+        <v>12.1</v>
       </c>
       <c r="K99" s="14" t="n">
         <v>5.8</v>
@@ -7187,7 +7187,7 @@
         <v>0</v>
       </c>
       <c r="D100" s="14" t="n">
-        <v>17.08</v>
+        <v>16.9</v>
       </c>
       <c r="E100" s="14" t="n">
         <v>0</v>
@@ -7205,7 +7205,7 @@
         <v>16.7</v>
       </c>
       <c r="J100" s="14" t="n">
-        <v>8.16</v>
+        <v>8.44</v>
       </c>
       <c r="K100" s="14" t="n">
         <v>3.4</v>
@@ -7250,7 +7250,7 @@
         <v>6.3</v>
       </c>
       <c r="D101" s="14" t="n">
-        <v>6.7</v>
+        <v>6.84</v>
       </c>
       <c r="E101" s="14" t="n">
         <v>7.8</v>
@@ -44213,7 +44213,7 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -44231,7 +44231,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -44257,7 +44257,7 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0.08</v>
+        <v>0.07</v>
       </c>
       <c r="D9" t="n">
         <v>0.08</v>
@@ -44275,7 +44275,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="J9" t="n">
         <v>0.02</v>
@@ -44301,7 +44301,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -44345,7 +44345,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="D11" t="n">
         <v>0.06</v>
@@ -44363,7 +44363,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J11" t="n">
         <v>0.01</v>
@@ -44389,7 +44389,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="D12" t="n">
         <v>0.05</v>
@@ -44433,7 +44433,7 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -44451,7 +44451,7 @@
         <v>0.09</v>
       </c>
       <c r="I13" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="J13" t="n">
         <v>0.05</v>
@@ -46255,7 +46255,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1.3</v>
+        <v>1.24</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -46281,7 +46281,7 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>2.38</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -46299,7 +46299,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -46325,7 +46325,7 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>1.62</v>
+        <v>1.4</v>
       </c>
       <c r="D9" t="n">
         <v>1.3</v>
@@ -46343,7 +46343,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2.92</v>
+        <v>3.06</v>
       </c>
       <c r="J9" t="n">
         <v>0.8</v>
@@ -46369,7 +46369,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>6.34</v>
+        <v>6.26</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -46387,7 +46387,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>6.3</v>
+        <v>6.26</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -46413,7 +46413,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>10.46</v>
+        <v>12.38</v>
       </c>
       <c r="D11" t="n">
         <v>1.1</v>
@@ -46431,7 +46431,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>10.34</v>
+        <v>7.18</v>
       </c>
       <c r="J11" t="n">
         <v>0.6</v>
@@ -46457,7 +46457,7 @@
         <v>0</v>
       </c>
       <c r="C12" t="n">
-        <v>10.84</v>
+        <v>10.88</v>
       </c>
       <c r="D12" t="n">
         <v>1.1</v>
@@ -46475,7 +46475,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>12.12</v>
+        <v>12.2</v>
       </c>
       <c r="J12" t="n">
         <v>1.1</v>
@@ -46501,7 +46501,7 @@
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>12.74</v>
+        <v>12.62</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -46519,7 +46519,7 @@
         <v>6.7</v>
       </c>
       <c r="I13" t="n">
-        <v>17.48</v>
+        <v>18.12</v>
       </c>
       <c r="J13" t="n">
         <v>2.8</v>
@@ -46545,7 +46545,7 @@
         <v>19.4</v>
       </c>
       <c r="C14" t="n">
-        <v>5.02</v>
+        <v>6.46</v>
       </c>
       <c r="D14" t="n">
         <v>1.8</v>
@@ -46563,7 +46563,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>15</v>
+        <v>12.1</v>
       </c>
       <c r="J14" t="n">
         <v>5.8</v>
@@ -46589,7 +46589,7 @@
         <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>17.08</v>
+        <v>16.9</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -46607,7 +46607,7 @@
         <v>16.7</v>
       </c>
       <c r="I15" t="n">
-        <v>8.16</v>
+        <v>8.44</v>
       </c>
       <c r="J15" t="n">
         <v>3.4</v>
@@ -46633,7 +46633,7 @@
         <v>6.3</v>
       </c>
       <c r="C16" t="n">
-        <v>6.7</v>
+        <v>6.84</v>
       </c>
       <c r="D16" t="n">
         <v>7.8</v>

</xml_diff>